<commit_message>
Add top-10 call sheet with contacts verified on official sites
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013pAYVPcDWTLeuLdwVsKmmQ
</commit_message>
<xml_diff>
--- a/suppliers_us/US_factories_check_2026-10-15.xlsx
+++ b/suppliers_us/US_factories_check_2026-10-15.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Заводы США 15.10" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Как проверено" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Обзвон топ-10" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Заводы США 15.10" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Как проверено" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -93,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -120,6 +121,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -485,6 +487,586 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Завод</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Город</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Телефон (с офиц. сайта)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Почта (с офиц. сайта)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Сайт</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>NSF 455-2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Зачем звонить</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Главный вопрос</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Результат звонка</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Health Genesis Corporation</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Дейви, FL, ~30 мин</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>(305) 861-0898; 800-595-6593</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>sales@healthgenesis.com</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>healthgenesis.com</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>да, 2 площадки</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>600+ готовых формул, пробиотики, рядом</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Какие из 4 позиций есть на складе и срок от утверждения этикетки до готовых банок</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Sun Nutraceuticals</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Форт-Лодердейл, FL, ~30 мин</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>(754) 247-9542</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>sales@sunnutra.com</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>sunnutra.com</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>нет (заявляют SGS GMP)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>колострум, магний, креатин на складе, 2-3 недели</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Срок от утверждения этикетки; номер сертификата SGS</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Natural Vitamins Laboratory (NV Labs)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Опа-Лока, FL, ~20 мин</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>305-265-1660</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>info@nvlabs.net</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>nvlabs.net</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>да, полный набор технологий</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>свои капсулы и порошки, ближе всех</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Какие из 4 позиций есть на складе и срок от утверждения этикетки до готовых банок</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Arnet Pharmaceutical</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Дейви, FL, ~30 мин</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>+1 (954) 236-9053; 800-968-6673</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>info@arnetusa.com</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>arnetusa.com</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>капсулы, смешивание, таблетки</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Какие из 4 позиций есть на складе и срок от утверждения этикетки до готовых банок</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ASAP Nutrition</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Форт-Лодердейл, FL, ~30 мин</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>+1 954-676-7058</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>partner@asapnutrition.us</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>asapnutrition.us</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>капсулы, порошки, смешивание</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Какие из 4 позиций есть на складе и срок от утверждения этикетки до готовых банок</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>FAME Health Labs</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Сидартаун, GA</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>+1 877-222-3530</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>partnerships@famehealthlabs.com</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>famehealthlabs.com</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>да, плюс SQF</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>сток от 500 банок</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Срок от утверждения этикетки; срок на первый заказ</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Your Gummy Vitamins</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Уэстон, FL, ~35 мин</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>(954) 306-6391</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>hello@YourGummyVitamins.com</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>yourgummyvitamins.com</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>да, есть капсулирование</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>от 500 единиц, быстрые сроки</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Срок от утверждения этикетки; делают ли капсулы, не только гуммис</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>BL Bio Lab</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Клируотер, FL</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>(727) 877-9889</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>почта на сайте не опубликована</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>blbiolab.com</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>да, полный набор</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>полный цикл</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Срок от утверждения этикетки; сроки: в обзорах 8-12 недель на новый продукт</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Vireo Systems</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Нэшвилл, TN</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>1-855-442-6466</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>info@vireosystems.com</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>vireosystems.com</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>креатин: свой патент на креатин HCl</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Срок от утверждения этикетки; только по креатину</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>ViaCore Nutrition</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Эль-Рино, OK</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>(405) 622-5123</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>почта на сайте не опубликована</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>viacorenutrition.com</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>готовый креатин от 48 банок</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Срок от утверждения этикетки; только по креатину</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Не звонить:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Vitamix Labs: предупреждение FDA от 20.04.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Nutra Group: сайт не работает, похоже на посредника</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Custom Nutra: только офис продаж, производства в реестре нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Alfa Vitamins Laboratories: нет официального сайта, телефон не подтвердить</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Ion Labs: сайт не открывается, в 2011 было предупреждение FDA</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1071,7 +1653,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>